<commit_message>
Done to fix bug
</commit_message>
<xml_diff>
--- a/output/DANHSACHGIAMSAT_ca1.XLSX
+++ b/output/DANHSACHGIAMSAT_ca1.XLSX
@@ -146,17 +146,157 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t/>
+          <t>101170089</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t/>
+          <t>Nguyễn Văn Cường</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Không có cán bộ giám sát</t>
+          <t>151</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>101170021</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Trần Vĩnh Hảo</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>222</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>3.0</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>101170047</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Hà Minh Phúc</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>165</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>4.0</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>101170039</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Văn Nhật Nam</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>187</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>101170024</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Võ Đăng Hiếu</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>201</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>6.0</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>101170186</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Bá Khải</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>178</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>7.0</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>101170182</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Nguyễn Tấn Hưng</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>161</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>8.0</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>101170172</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Hồ Minh Đạt</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>189</t>
         </is>
       </c>
     </row>

</xml_diff>